<commit_message>
lka events can be extracted
</commit_message>
<xml_diff>
--- a/config/kpi_as_lat.xlsx
+++ b/config/kpi_as_lat.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wangjianhai/02_ADAS/01_repo/01_Tools/01_kpi_extractor/python/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77FE6299-BD87-DD4E-9441-D160095415BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D12CD59-A666-AC4A-82AD-8BD4246004EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="700" windowWidth="34200" windowHeight="20360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34220" yWindow="7000" windowWidth="38400" windowHeight="14600" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="paramASLat" sheetId="7" r:id="rId1"/>
-    <sheet name="graphASLat" sheetId="3" r:id="rId2"/>
-    <sheet name="kpiASLat" sheetId="6" r:id="rId3"/>
+    <sheet name="paramAsLat" sheetId="7" r:id="rId1"/>
+    <sheet name="graphAsLat" sheetId="3" r:id="rId2"/>
+    <sheet name="kpiAsLat" sheetId="6" r:id="rId3"/>
     <sheet name="markerShapes" sheetId="5" r:id="rId4"/>
     <sheet name="lineColors" sheetId="4" r:id="rId5"/>
   </sheets>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="57">
   <si>
     <t>Reference</t>
   </si>
@@ -170,6 +170,45 @@
   </si>
   <si>
     <t>Class</t>
+  </si>
+  <si>
+    <t>LKA</t>
+  </si>
+  <si>
+    <t>double</t>
+  </si>
+  <si>
+    <t>m</t>
+  </si>
+  <si>
+    <t>isWhlTrqHigh</t>
+  </si>
+  <si>
+    <t>bool</t>
+  </si>
+  <si>
+    <t>Driver_Interaction_Torque</t>
+  </si>
+  <si>
+    <t>float</t>
+  </si>
+  <si>
+    <t>Nm</t>
+  </si>
+  <si>
+    <t>The torque which it is considered the driver to be resisting the intervention</t>
+  </si>
+  <si>
+    <t>LkaEventDetector</t>
+  </si>
+  <si>
+    <t>MinDTLEDelta</t>
+  </si>
+  <si>
+    <t>Difference between target DTLE and actual min dtle</t>
+  </si>
+  <si>
+    <t>steering wheel torque is above Driver_Interaction_Torque</t>
   </si>
 </sst>
 </file>
@@ -609,7 +648,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6ECBDC44-4FC0-EE44-827D-4641F2FAC044}">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -636,6 +675,26 @@
       </c>
       <c r="F1" s="5" t="s">
         <v>43</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F2" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -992,20 +1051,38 @@
       </c>
     </row>
     <row r="2" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
+      <c r="B2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E2" t="s">
+        <v>46</v>
+      </c>
+      <c r="F2"/>
+      <c r="G2" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="3" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B3" s="12"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
+      <c r="B3" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>48</v>
+      </c>
       <c r="E3" s="12"/>
       <c r="F3" s="12"/>
-      <c r="G3" s="12"/>
+      <c r="G3" s="12" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B4" s="12"/>

</xml_diff>

<commit_message>
adaptive file generation + lka kpi extracted
</commit_message>
<xml_diff>
--- a/config/kpi_as_lat.xlsx
+++ b/config/kpi_as_lat.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wangjianhai/02_ADAS/01_repo/01_Tools/01_kpi_extractor/python/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D12CD59-A666-AC4A-82AD-8BD4246004EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FC74FC8-12B7-6745-9F45-5685C01354AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34220" yWindow="7000" windowWidth="38400" windowHeight="14600" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34200" yWindow="7000" windowWidth="38400" windowHeight="14600" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="paramAsLat" sheetId="7" r:id="rId1"/>
-    <sheet name="graphAsLat" sheetId="3" r:id="rId2"/>
-    <sheet name="kpiAsLat" sheetId="6" r:id="rId3"/>
+    <sheet name="params" sheetId="7" r:id="rId1"/>
+    <sheet name="graphSpec" sheetId="3" r:id="rId2"/>
+    <sheet name="KPI" sheetId="6" r:id="rId3"/>
     <sheet name="markerShapes" sheetId="5" r:id="rId4"/>
     <sheet name="lineColors" sheetId="4" r:id="rId5"/>
   </sheets>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="64">
   <si>
     <t>Reference</t>
   </si>
@@ -205,10 +205,31 @@
     <t>MinDTLEDelta</t>
   </si>
   <si>
-    <t>Difference between target DTLE and actual min dtle</t>
-  </si>
-  <si>
-    <t>steering wheel torque is above Driver_Interaction_Torque</t>
+    <t>Common</t>
+  </si>
+  <si>
+    <t>label</t>
+  </si>
+  <si>
+    <t>string</t>
+  </si>
+  <si>
+    <t>name of the mdf chunk</t>
+  </si>
+  <si>
+    <t>logTime</t>
+  </si>
+  <si>
+    <t>Logging time since recording start</t>
+  </si>
+  <si>
+    <t>vehSpd</t>
+  </si>
+  <si>
+    <t>kph</t>
+  </si>
+  <si>
+    <t>Vehicle speed at time of event</t>
   </si>
 </sst>
 </file>
@@ -1017,7 +1038,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CE39B99-0AFB-8547-83BF-D855CC6E3BB3}">
-  <dimension ref="B1:G43"/>
+  <dimension ref="B1:G46"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2.83203125" style="13" customWidth="1"/>
@@ -1051,59 +1072,83 @@
       </c>
     </row>
     <row r="2" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C2" t="s">
-        <v>54</v>
-      </c>
-      <c r="D2" t="s">
-        <v>45</v>
-      </c>
-      <c r="E2" t="s">
-        <v>46</v>
-      </c>
-      <c r="F2"/>
-      <c r="G2" t="s">
+      <c r="B2" s="12" t="s">
         <v>55</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B3" s="12" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="E3" s="12"/>
+        <v>45</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>14</v>
+      </c>
       <c r="F3" s="12"/>
       <c r="G3" s="12" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B4" s="12"/>
-      <c r="C4" s="12"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="12"/>
+      <c r="B4" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>62</v>
+      </c>
       <c r="F4" s="12"/>
-      <c r="G4" s="12"/>
+      <c r="G4" s="12" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B5" s="12"/>
-      <c r="C5" s="12"/>
-      <c r="D5" s="12"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="12"/>
+      <c r="B5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C5" t="s">
+        <v>54</v>
+      </c>
+      <c r="D5" t="s">
+        <v>45</v>
+      </c>
+      <c r="E5" t="s">
+        <v>46</v>
+      </c>
+      <c r="F5"/>
       <c r="G5" s="12"/>
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B6" s="12"/>
-      <c r="C6" s="12"/>
-      <c r="D6" s="12"/>
+      <c r="B6" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>48</v>
+      </c>
       <c r="E6" s="12"/>
       <c r="F6" s="12"/>
       <c r="G6" s="12"/>
@@ -1297,6 +1342,7 @@
       <c r="C30" s="12"/>
       <c r="D30" s="12"/>
       <c r="E30" s="12"/>
+      <c r="F30" s="12"/>
       <c r="G30" s="12"/>
     </row>
     <row r="31" spans="2:7" x14ac:dyDescent="0.2">
@@ -1320,7 +1366,6 @@
       <c r="C33" s="12"/>
       <c r="D33" s="12"/>
       <c r="E33" s="12"/>
-      <c r="F33" s="12"/>
       <c r="G33" s="12"/>
     </row>
     <row r="34" spans="2:7" x14ac:dyDescent="0.2">
@@ -1352,6 +1397,7 @@
       <c r="C37" s="12"/>
       <c r="D37" s="12"/>
       <c r="E37" s="12"/>
+      <c r="F37" s="12"/>
       <c r="G37" s="12"/>
     </row>
     <row r="38" spans="2:7" x14ac:dyDescent="0.2">
@@ -1359,6 +1405,7 @@
       <c r="C38" s="12"/>
       <c r="D38" s="12"/>
       <c r="E38" s="12"/>
+      <c r="F38" s="12"/>
       <c r="G38" s="12"/>
     </row>
     <row r="39" spans="2:7" x14ac:dyDescent="0.2">
@@ -1366,6 +1413,7 @@
       <c r="C39" s="12"/>
       <c r="D39" s="12"/>
       <c r="E39" s="12"/>
+      <c r="F39" s="12"/>
       <c r="G39" s="12"/>
     </row>
     <row r="40" spans="2:7" x14ac:dyDescent="0.2">
@@ -1394,8 +1442,26 @@
       <c r="C43" s="12"/>
       <c r="D43" s="12"/>
       <c r="E43" s="12"/>
-      <c r="F43" s="14"/>
       <c r="G43" s="12"/>
+    </row>
+    <row r="44" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B44" s="12"/>
+      <c r="C44" s="12"/>
+      <c r="D44" s="12"/>
+      <c r="E44" s="12"/>
+    </row>
+    <row r="45" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B45" s="12"/>
+      <c r="C45" s="12"/>
+      <c r="D45" s="12"/>
+      <c r="E45" s="12"/>
+    </row>
+    <row r="46" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B46" s="12"/>
+      <c r="C46" s="12"/>
+      <c r="D46" s="12"/>
+      <c r="E46" s="12"/>
+      <c r="F46" s="14"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
lka scatter can be generated but only isWhlTrqHigh can be plotted
</commit_message>
<xml_diff>
--- a/config/kpi_as_lat.xlsx
+++ b/config/kpi_as_lat.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wangjianhai/02_ADAS/01_repo/01_Tools/01_kpi_extractor/python/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FC74FC8-12B7-6745-9F45-5685C01354AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ACC31AD-EE20-3C4E-8BF0-FE2207E0125A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34200" yWindow="7000" windowWidth="38400" windowHeight="14600" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38340" yWindow="6380" windowWidth="38400" windowHeight="14600" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="params" sheetId="7" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="73">
   <si>
     <t>Reference</t>
   </si>
@@ -230,6 +230,33 @@
   </si>
   <si>
     <t>Vehicle speed at time of event</t>
+  </si>
+  <si>
+    <t>Common_x</t>
+  </si>
+  <si>
+    <t>Ego Speed</t>
+  </si>
+  <si>
+    <t>Ego Speed (km/h)</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>none</t>
+  </si>
+  <si>
+    <t>scatter</t>
+  </si>
+  <si>
+    <t>Distance (m)</t>
+  </si>
+  <si>
+    <t>Difference: lane-edge target vs. achieved minimum</t>
+  </si>
+  <si>
+    <t>MinDTLEDlta</t>
   </si>
 </sst>
 </file>
@@ -736,7 +763,7 @@
     <col min="5" max="5" width="13.5" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="22" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="20.83203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="26.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17" customWidth="1"/>
     <col min="9" max="9" width="36.83203125" customWidth="1"/>
     <col min="11" max="11" width="15.5" customWidth="1"/>
   </cols>
@@ -780,32 +807,80 @@
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
-      <c r="L2" s="1"/>
+      <c r="A2" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D2" s="2">
+        <v>0</v>
+      </c>
+      <c r="E2" s="2">
+        <v>120</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="K2" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L2" s="1" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
-      <c r="K3" s="1"/>
-      <c r="L3" s="1"/>
+      <c r="A3" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D3" s="2">
+        <v>-3</v>
+      </c>
+      <c r="E3" s="2">
+        <v>3</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="K3" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L3" s="1" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>

</xml_diff>

<commit_message>
add as long signals for availability check
</commit_message>
<xml_diff>
--- a/config/kpi_as_lat.xlsx
+++ b/config/kpi_as_lat.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wangjianhai/02_ADAS/01_repo/01_Tools/01_kpi_extractor/python/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EABD6DB-7A5F-6C4E-B1ED-465889D3C819}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{033D4CE4-1EB1-E140-AC93-796B4A7B4BDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="700" windowWidth="34200" windowHeight="20520" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="700" windowWidth="34200" windowHeight="20460" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="params" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="124">
   <si>
     <t>Parameter</t>
   </si>
@@ -1252,9 +1252,6 @@
       <c r="C2" t="s">
         <v>52</v>
       </c>
-      <c r="F2" t="s">
-        <v>53</v>
-      </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
@@ -1283,9 +1280,6 @@
       <c r="E4" t="s">
         <v>61</v>
       </c>
-      <c r="F4" t="s">
-        <v>62</v>
-      </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
@@ -1302,9 +1296,6 @@
       </c>
       <c r="E5" t="s">
         <v>61</v>
-      </c>
-      <c r="F5" t="s">
-        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>